<commit_message>
resolved problem with prices overload
</commit_message>
<xml_diff>
--- a/public/upload_templates/price_template.xlsx
+++ b/public/upload_templates/price_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\albabello\erp_app\public\upload_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3A92027-5B9E-423F-AC2C-0CEB44FE6AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042933F1-4866-4B5D-8601-B7D50517AE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{755590B0-EA17-435E-B3C3-7014BD156F2B}"/>
   </bookViews>
@@ -34,14 +34,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>product_code</t>
   </si>
   <si>
-    <t>selling_price</t>
-  </si>
-  <si>
     <t>CZ0180063</t>
   </si>
   <si>
@@ -52,6 +49,12 @@
   </si>
   <si>
     <t>cost_price</t>
+  </si>
+  <si>
+    <t>retail_price</t>
+  </si>
+  <si>
+    <t>whole_price</t>
   </si>
 </sst>
 </file>
@@ -403,27 +406,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077B09B4-9258-43CD-862C-873F19ED84D3}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
+      <c r="D1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2">
         <v>12000</v>
@@ -431,10 +437,13 @@
       <c r="C2">
         <v>13000</v>
       </c>
+      <c r="D2">
+        <v>12900</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>17580</v>
@@ -442,16 +451,22 @@
       <c r="C3">
         <v>18100</v>
       </c>
+      <c r="D3">
+        <v>18000</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>4450</v>
       </c>
       <c r="C4">
         <v>4500</v>
+      </c>
+      <c r="D4">
+        <v>4450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>